<commit_message>
📊 NY session — 2026-08-25
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q93"/>
+  <dimension ref="A1:Q94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6221,6 +6221,67 @@
       </c>
       <c r="Q93" s="19" t="inlineStr"/>
     </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B94" s="15" t="inlineStr">
+        <is>
+          <t>20:58:43</t>
+        </is>
+      </c>
+      <c r="C94" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E94" s="15" t="n">
+        <v>4615.22</v>
+      </c>
+      <c r="F94" s="15" t="n">
+        <v>4627.68</v>
+      </c>
+      <c r="G94" s="15" t="n">
+        <v>4596.52</v>
+      </c>
+      <c r="H94" s="15" t="n">
+        <v>4590.29</v>
+      </c>
+      <c r="I94" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J94" s="15" t="n">
+        <v>4642.29</v>
+      </c>
+      <c r="K94" s="18" t="n">
+        <v>-27070</v>
+      </c>
+      <c r="L94" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M94" s="18" t="n">
+        <v>-27070.05</v>
+      </c>
+      <c r="N94" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q94" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6237,7 +6298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q79"/>
+  <dimension ref="A1:Q80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10995,6 +11056,67 @@
         </is>
       </c>
       <c r="Q79" s="24" t="inlineStr"/>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>20:58:43</t>
+        </is>
+      </c>
+      <c r="C80" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D80" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E80" s="15" t="n">
+        <v>4615.22</v>
+      </c>
+      <c r="F80" s="15" t="n">
+        <v>4627.68</v>
+      </c>
+      <c r="G80" s="15" t="n">
+        <v>4596.52</v>
+      </c>
+      <c r="H80" s="15" t="n">
+        <v>4590.29</v>
+      </c>
+      <c r="I80" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J80" s="15" t="n">
+        <v>4642.29</v>
+      </c>
+      <c r="K80" s="18" t="n">
+        <v>-27070</v>
+      </c>
+      <c r="L80" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M80" s="18" t="n">
+        <v>-27070.05</v>
+      </c>
+      <c r="N80" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q80" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-08-26
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q94"/>
+  <dimension ref="A1:Q95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6282,6 +6282,67 @@
       </c>
       <c r="Q94" s="19" t="inlineStr"/>
     </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B95" s="20" t="inlineStr">
+        <is>
+          <t>18:46:21</t>
+        </is>
+      </c>
+      <c r="C95" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D95" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E95" s="20" t="n">
+        <v>4620.9</v>
+      </c>
+      <c r="F95" s="20" t="n">
+        <v>4631.87</v>
+      </c>
+      <c r="G95" s="20" t="n">
+        <v>4604.45</v>
+      </c>
+      <c r="H95" s="20" t="n">
+        <v>4598.96</v>
+      </c>
+      <c r="I95" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J95" s="20" t="n">
+        <v>4599.85</v>
+      </c>
+      <c r="K95" s="23" t="n">
+        <v>21050</v>
+      </c>
+      <c r="L95" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M95" s="23" t="n">
+        <v>21049.95</v>
+      </c>
+      <c r="N95" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q95" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6298,7 +6359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q80"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11117,6 +11178,67 @@
         </is>
       </c>
       <c r="Q80" s="19" t="inlineStr"/>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B81" s="20" t="inlineStr">
+        <is>
+          <t>18:46:21</t>
+        </is>
+      </c>
+      <c r="C81" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E81" s="20" t="n">
+        <v>4620.9</v>
+      </c>
+      <c r="F81" s="20" t="n">
+        <v>4631.87</v>
+      </c>
+      <c r="G81" s="20" t="n">
+        <v>4604.45</v>
+      </c>
+      <c r="H81" s="20" t="n">
+        <v>4598.96</v>
+      </c>
+      <c r="I81" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J81" s="20" t="n">
+        <v>4599.85</v>
+      </c>
+      <c r="K81" s="23" t="n">
+        <v>21050</v>
+      </c>
+      <c r="L81" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M81" s="23" t="n">
+        <v>21049.95</v>
+      </c>
+      <c r="N81" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q81" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 NY session — 2026-08-26
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q95"/>
+  <dimension ref="A1:Q97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6343,6 +6343,128 @@
       </c>
       <c r="Q95" s="24" t="inlineStr"/>
     </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B96" s="20" t="inlineStr">
+        <is>
+          <t>21:36:02</t>
+        </is>
+      </c>
+      <c r="C96" s="23" t="inlineStr">
+        <is>
+          <t>S2 Goldmine</t>
+        </is>
+      </c>
+      <c r="D96" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E96" s="20" t="n">
+        <v>4625.56</v>
+      </c>
+      <c r="F96" s="20" t="n">
+        <v>4640.5</v>
+      </c>
+      <c r="G96" s="20" t="n">
+        <v>4603.15</v>
+      </c>
+      <c r="H96" s="20" t="n">
+        <v>4595.69</v>
+      </c>
+      <c r="I96" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J96" s="20" t="n">
+        <v>4601.18</v>
+      </c>
+      <c r="K96" s="23" t="n">
+        <v>24380</v>
+      </c>
+      <c r="L96" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M96" s="23" t="n">
+        <v>24379.95</v>
+      </c>
+      <c r="N96" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q96" s="24" t="inlineStr"/>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B97" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C97" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D97" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E97" s="20" t="n">
+        <v>4596.19</v>
+      </c>
+      <c r="F97" s="20" t="n">
+        <v>4610.03</v>
+      </c>
+      <c r="G97" s="20" t="n">
+        <v>4575.44</v>
+      </c>
+      <c r="H97" s="20" t="n">
+        <v>4568.52</v>
+      </c>
+      <c r="I97" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J97" s="20" t="n">
+        <v>4594.15</v>
+      </c>
+      <c r="K97" s="23" t="n">
+        <v>2040</v>
+      </c>
+      <c r="L97" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M97" s="23" t="n">
+        <v>2039.95</v>
+      </c>
+      <c r="N97" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P97" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q97" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6359,7 +6481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q81"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11240,6 +11362,67 @@
       </c>
       <c r="Q81" s="24" t="inlineStr"/>
     </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B82" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C82" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D82" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E82" s="20" t="n">
+        <v>4596.19</v>
+      </c>
+      <c r="F82" s="20" t="n">
+        <v>4610.03</v>
+      </c>
+      <c r="G82" s="20" t="n">
+        <v>4575.44</v>
+      </c>
+      <c r="H82" s="20" t="n">
+        <v>4568.52</v>
+      </c>
+      <c r="I82" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J82" s="20" t="n">
+        <v>4594.15</v>
+      </c>
+      <c r="K82" s="23" t="n">
+        <v>2040</v>
+      </c>
+      <c r="L82" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M82" s="23" t="n">
+        <v>2039.95</v>
+      </c>
+      <c r="N82" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q82" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -11256,7 +11439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11683,6 +11866,67 @@
         </is>
       </c>
       <c r="Q8" s="24" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>21:36:02</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>S2 Goldmine</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>4625.56</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>4640.5</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>4603.15</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>4595.69</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <v>4601.18</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <v>24380</v>
+      </c>
+      <c r="L9" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M9" s="23" t="n">
+        <v>24379.95</v>
+      </c>
+      <c r="N9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q9" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-02
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q97"/>
+  <dimension ref="A1:Q99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6465,6 +6465,128 @@
       </c>
       <c r="Q97" s="24" t="inlineStr"/>
     </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B98" s="20" t="inlineStr">
+        <is>
+          <t>17:49:38</t>
+        </is>
+      </c>
+      <c r="C98" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D98" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E98" s="20" t="n">
+        <v>4338.5</v>
+      </c>
+      <c r="F98" s="20" t="n">
+        <v>4351.83</v>
+      </c>
+      <c r="G98" s="20" t="n">
+        <v>4318.52</v>
+      </c>
+      <c r="H98" s="20" t="n">
+        <v>4311.85</v>
+      </c>
+      <c r="I98" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J98" s="20" t="n">
+        <v>4333.38</v>
+      </c>
+      <c r="K98" s="23" t="n">
+        <v>5125</v>
+      </c>
+      <c r="L98" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M98" s="23" t="n">
+        <v>5124.95</v>
+      </c>
+      <c r="N98" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q98" s="24" t="inlineStr"/>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B99" s="20" t="inlineStr">
+        <is>
+          <t>19:13:31</t>
+        </is>
+      </c>
+      <c r="C99" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D99" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E99" s="20" t="n">
+        <v>4346.71</v>
+      </c>
+      <c r="F99" s="20" t="n">
+        <v>4332.26</v>
+      </c>
+      <c r="G99" s="20" t="n">
+        <v>4368.39</v>
+      </c>
+      <c r="H99" s="20" t="n">
+        <v>4375.61</v>
+      </c>
+      <c r="I99" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J99" s="20" t="n">
+        <v>4369.93</v>
+      </c>
+      <c r="K99" s="23" t="n">
+        <v>23215</v>
+      </c>
+      <c r="L99" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M99" s="23" t="n">
+        <v>23214.95</v>
+      </c>
+      <c r="N99" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q99" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6481,7 +6603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q82"/>
+  <dimension ref="A1:Q84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11422,6 +11544,128 @@
         </is>
       </c>
       <c r="Q82" s="24" t="inlineStr"/>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B83" s="20" t="inlineStr">
+        <is>
+          <t>17:49:38</t>
+        </is>
+      </c>
+      <c r="C83" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E83" s="20" t="n">
+        <v>4338.5</v>
+      </c>
+      <c r="F83" s="20" t="n">
+        <v>4351.83</v>
+      </c>
+      <c r="G83" s="20" t="n">
+        <v>4318.52</v>
+      </c>
+      <c r="H83" s="20" t="n">
+        <v>4311.85</v>
+      </c>
+      <c r="I83" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J83" s="20" t="n">
+        <v>4333.38</v>
+      </c>
+      <c r="K83" s="23" t="n">
+        <v>5125</v>
+      </c>
+      <c r="L83" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M83" s="23" t="n">
+        <v>5124.95</v>
+      </c>
+      <c r="N83" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P83" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q83" s="24" t="inlineStr"/>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B84" s="20" t="inlineStr">
+        <is>
+          <t>19:13:31</t>
+        </is>
+      </c>
+      <c r="C84" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D84" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E84" s="20" t="n">
+        <v>4346.71</v>
+      </c>
+      <c r="F84" s="20" t="n">
+        <v>4332.26</v>
+      </c>
+      <c r="G84" s="20" t="n">
+        <v>4368.39</v>
+      </c>
+      <c r="H84" s="20" t="n">
+        <v>4375.61</v>
+      </c>
+      <c r="I84" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J84" s="20" t="n">
+        <v>4369.93</v>
+      </c>
+      <c r="K84" s="23" t="n">
+        <v>23215</v>
+      </c>
+      <c r="L84" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M84" s="23" t="n">
+        <v>23214.95</v>
+      </c>
+      <c r="N84" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P84" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q84" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-09
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q99"/>
+  <dimension ref="A1:Q101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6587,6 +6587,128 @@
       </c>
       <c r="Q99" s="24" t="inlineStr"/>
     </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B100" s="20" t="inlineStr">
+        <is>
+          <t>18:01:21</t>
+        </is>
+      </c>
+      <c r="C100" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D100" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E100" s="20" t="n">
+        <v>4403.06</v>
+      </c>
+      <c r="F100" s="20" t="n">
+        <v>4418.67</v>
+      </c>
+      <c r="G100" s="20" t="n">
+        <v>4379.65</v>
+      </c>
+      <c r="H100" s="20" t="n">
+        <v>4371.85</v>
+      </c>
+      <c r="I100" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J100" s="20" t="n">
+        <v>4393.82</v>
+      </c>
+      <c r="K100" s="23" t="n">
+        <v>9235</v>
+      </c>
+      <c r="L100" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M100" s="23" t="n">
+        <v>9234.950000000001</v>
+      </c>
+      <c r="N100" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P100" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q100" s="24" t="inlineStr"/>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B101" s="15" t="inlineStr">
+        <is>
+          <t>22:33:12</t>
+        </is>
+      </c>
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D101" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E101" s="15" t="n">
+        <v>4391.73</v>
+      </c>
+      <c r="F101" s="15" t="n">
+        <v>4414.3</v>
+      </c>
+      <c r="G101" s="15" t="n">
+        <v>4357.86</v>
+      </c>
+      <c r="H101" s="15" t="n">
+        <v>4346.57</v>
+      </c>
+      <c r="I101" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J101" s="15" t="n">
+        <v>4413.43</v>
+      </c>
+      <c r="K101" s="18" t="n">
+        <v>-21705</v>
+      </c>
+      <c r="L101" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M101" s="18" t="n">
+        <v>-21705.05</v>
+      </c>
+      <c r="N101" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q101" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6603,7 +6725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q84"/>
+  <dimension ref="A1:Q85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11666,6 +11788,67 @@
         </is>
       </c>
       <c r="Q84" s="24" t="inlineStr"/>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B85" s="20" t="inlineStr">
+        <is>
+          <t>18:01:21</t>
+        </is>
+      </c>
+      <c r="C85" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D85" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E85" s="20" t="n">
+        <v>4403.06</v>
+      </c>
+      <c r="F85" s="20" t="n">
+        <v>4418.67</v>
+      </c>
+      <c r="G85" s="20" t="n">
+        <v>4379.65</v>
+      </c>
+      <c r="H85" s="20" t="n">
+        <v>4371.85</v>
+      </c>
+      <c r="I85" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J85" s="20" t="n">
+        <v>4393.82</v>
+      </c>
+      <c r="K85" s="23" t="n">
+        <v>9235</v>
+      </c>
+      <c r="L85" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M85" s="23" t="n">
+        <v>9234.950000000001</v>
+      </c>
+      <c r="N85" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q85" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -12188,7 +12371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12859,6 +13042,67 @@
         </is>
       </c>
       <c r="Q12" s="19" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>22:33:12</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>4391.73</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>4414.3</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>4357.86</v>
+      </c>
+      <c r="H13" s="15" t="n">
+        <v>4346.57</v>
+      </c>
+      <c r="I13" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J13" s="15" t="n">
+        <v>4413.43</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>-21705</v>
+      </c>
+      <c r="L13" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M13" s="18" t="n">
+        <v>-21705.05</v>
+      </c>
+      <c r="N13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q13" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-15
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q101"/>
+  <dimension ref="A1:Q103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6709,6 +6709,128 @@
       </c>
       <c r="Q101" s="19" t="inlineStr"/>
     </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B102" s="20" t="inlineStr">
+        <is>
+          <t>18:25:55</t>
+        </is>
+      </c>
+      <c r="C102" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D102" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E102" s="20" t="n">
+        <v>4348.55</v>
+      </c>
+      <c r="F102" s="20" t="n">
+        <v>4362.53</v>
+      </c>
+      <c r="G102" s="20" t="n">
+        <v>4327.56</v>
+      </c>
+      <c r="H102" s="20" t="n">
+        <v>4320.57</v>
+      </c>
+      <c r="I102" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J102" s="20" t="n">
+        <v>4292.36</v>
+      </c>
+      <c r="K102" s="23" t="n">
+        <v>56180</v>
+      </c>
+      <c r="L102" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M102" s="23" t="n">
+        <v>56179.95</v>
+      </c>
+      <c r="N102" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q102" s="24" t="inlineStr"/>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B103" s="15" t="inlineStr">
+        <is>
+          <t>21:26:27</t>
+        </is>
+      </c>
+      <c r="C103" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D103" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E103" s="15" t="n">
+        <v>4282.04</v>
+      </c>
+      <c r="F103" s="15" t="n">
+        <v>4294.8</v>
+      </c>
+      <c r="G103" s="15" t="n">
+        <v>4262.89</v>
+      </c>
+      <c r="H103" s="15" t="n">
+        <v>4256.51</v>
+      </c>
+      <c r="I103" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J103" s="15" t="n">
+        <v>4291.97</v>
+      </c>
+      <c r="K103" s="18" t="n">
+        <v>-9925</v>
+      </c>
+      <c r="L103" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M103" s="18" t="n">
+        <v>-9925.049999999999</v>
+      </c>
+      <c r="N103" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q103" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6725,7 +6847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q85"/>
+  <dimension ref="A1:Q87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11849,6 +11971,128 @@
         </is>
       </c>
       <c r="Q85" s="24" t="inlineStr"/>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B86" s="20" t="inlineStr">
+        <is>
+          <t>18:25:55</t>
+        </is>
+      </c>
+      <c r="C86" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D86" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E86" s="20" t="n">
+        <v>4348.55</v>
+      </c>
+      <c r="F86" s="20" t="n">
+        <v>4362.53</v>
+      </c>
+      <c r="G86" s="20" t="n">
+        <v>4327.56</v>
+      </c>
+      <c r="H86" s="20" t="n">
+        <v>4320.57</v>
+      </c>
+      <c r="I86" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J86" s="20" t="n">
+        <v>4292.36</v>
+      </c>
+      <c r="K86" s="23" t="n">
+        <v>56180</v>
+      </c>
+      <c r="L86" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M86" s="23" t="n">
+        <v>56179.95</v>
+      </c>
+      <c r="N86" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q86" s="24" t="inlineStr"/>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>21:26:27</t>
+        </is>
+      </c>
+      <c r="C87" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E87" s="15" t="n">
+        <v>4282.04</v>
+      </c>
+      <c r="F87" s="15" t="n">
+        <v>4294.8</v>
+      </c>
+      <c r="G87" s="15" t="n">
+        <v>4262.89</v>
+      </c>
+      <c r="H87" s="15" t="n">
+        <v>4256.51</v>
+      </c>
+      <c r="I87" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J87" s="15" t="n">
+        <v>4291.97</v>
+      </c>
+      <c r="K87" s="18" t="n">
+        <v>-9925</v>
+      </c>
+      <c r="L87" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M87" s="18" t="n">
+        <v>-9925.049999999999</v>
+      </c>
+      <c r="N87" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q87" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-16
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q103"/>
+  <dimension ref="A1:Q104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6830,6 +6830,67 @@
         </is>
       </c>
       <c r="Q103" s="19" t="inlineStr"/>
+    </row>
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>23:31:33</t>
+        </is>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D104" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E104" s="15" t="n">
+        <v>4350.74</v>
+      </c>
+      <c r="F104" s="15" t="n">
+        <v>4334.47</v>
+      </c>
+      <c r="G104" s="15" t="n">
+        <v>4375.15</v>
+      </c>
+      <c r="H104" s="15" t="n">
+        <v>4383.28</v>
+      </c>
+      <c r="I104" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J104" s="15" t="n">
+        <v>4331.05</v>
+      </c>
+      <c r="K104" s="18" t="n">
+        <v>-19690</v>
+      </c>
+      <c r="L104" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M104" s="18" t="n">
+        <v>-19690.05</v>
+      </c>
+      <c r="N104" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P104" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q104" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -12615,7 +12676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13347,6 +13408,67 @@
         </is>
       </c>
       <c r="Q13" s="19" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>23:31:33</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>4350.74</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>4334.47</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>4375.15</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>4383.28</v>
+      </c>
+      <c r="I14" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J14" s="15" t="n">
+        <v>4331.05</v>
+      </c>
+      <c r="K14" s="18" t="n">
+        <v>-19690</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M14" s="18" t="n">
+        <v>-19690.05</v>
+      </c>
+      <c r="N14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q14" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-17
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q104"/>
+  <dimension ref="A1:Q105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6892,6 +6892,67 @@
       </c>
       <c r="Q104" s="19" t="inlineStr"/>
     </row>
+    <row r="105" ht="20" customHeight="1">
+      <c r="A105" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B105" s="15" t="inlineStr">
+        <is>
+          <t>00:05:16</t>
+        </is>
+      </c>
+      <c r="C105" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D105" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E105" s="15" t="n">
+        <v>4368.85</v>
+      </c>
+      <c r="F105" s="15" t="n">
+        <v>4350.13</v>
+      </c>
+      <c r="G105" s="15" t="n">
+        <v>4396.91</v>
+      </c>
+      <c r="H105" s="15" t="n">
+        <v>4406.27</v>
+      </c>
+      <c r="I105" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J105" s="15" t="n">
+        <v>4349.72</v>
+      </c>
+      <c r="K105" s="18" t="n">
+        <v>-19130</v>
+      </c>
+      <c r="L105" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M105" s="18" t="n">
+        <v>-19130.05</v>
+      </c>
+      <c r="N105" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q105" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6908,7 +6969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q87"/>
+  <dimension ref="A1:Q88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12154,6 +12215,67 @@
         </is>
       </c>
       <c r="Q87" s="19" t="inlineStr"/>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>00:05:16</t>
+        </is>
+      </c>
+      <c r="C88" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D88" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E88" s="15" t="n">
+        <v>4368.85</v>
+      </c>
+      <c r="F88" s="15" t="n">
+        <v>4350.13</v>
+      </c>
+      <c r="G88" s="15" t="n">
+        <v>4396.91</v>
+      </c>
+      <c r="H88" s="15" t="n">
+        <v>4406.27</v>
+      </c>
+      <c r="I88" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J88" s="15" t="n">
+        <v>4349.72</v>
+      </c>
+      <c r="K88" s="18" t="n">
+        <v>-19130</v>
+      </c>
+      <c r="L88" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M88" s="18" t="n">
+        <v>-19130.05</v>
+      </c>
+      <c r="N88" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O88" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q88" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-22
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q105"/>
+  <dimension ref="A1:Q106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6953,6 +6953,67 @@
       </c>
       <c r="Q105" s="19" t="inlineStr"/>
     </row>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>23:25:23</t>
+        </is>
+      </c>
+      <c r="C106" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D106" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E106" s="15" t="n">
+        <v>4337.46</v>
+      </c>
+      <c r="F106" s="15" t="n">
+        <v>4350.83</v>
+      </c>
+      <c r="G106" s="15" t="n">
+        <v>4317.4</v>
+      </c>
+      <c r="H106" s="15" t="n">
+        <v>4310.71</v>
+      </c>
+      <c r="I106" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J106" s="15" t="n">
+        <v>4349.03</v>
+      </c>
+      <c r="K106" s="18" t="n">
+        <v>-11570</v>
+      </c>
+      <c r="L106" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M106" s="18" t="n">
+        <v>-11570.05</v>
+      </c>
+      <c r="N106" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q106" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -6969,7 +7030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q88"/>
+  <dimension ref="A1:Q89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12276,6 +12337,67 @@
         </is>
       </c>
       <c r="Q88" s="19" t="inlineStr"/>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>23:25:23</t>
+        </is>
+      </c>
+      <c r="C89" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E89" s="15" t="n">
+        <v>4337.46</v>
+      </c>
+      <c r="F89" s="15" t="n">
+        <v>4350.83</v>
+      </c>
+      <c r="G89" s="15" t="n">
+        <v>4317.4</v>
+      </c>
+      <c r="H89" s="15" t="n">
+        <v>4310.71</v>
+      </c>
+      <c r="I89" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J89" s="15" t="n">
+        <v>4349.03</v>
+      </c>
+      <c r="K89" s="18" t="n">
+        <v>-11570</v>
+      </c>
+      <c r="L89" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M89" s="18" t="n">
+        <v>-11570.05</v>
+      </c>
+      <c r="N89" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q89" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-24
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q106"/>
+  <dimension ref="A1:Q108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7014,6 +7014,128 @@
       </c>
       <c r="Q106" s="19" t="inlineStr"/>
     </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B107" s="20" t="inlineStr">
+        <is>
+          <t>18:27:09</t>
+        </is>
+      </c>
+      <c r="C107" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D107" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E107" s="20" t="n">
+        <v>4289.75</v>
+      </c>
+      <c r="F107" s="20" t="n">
+        <v>4302.26</v>
+      </c>
+      <c r="G107" s="20" t="n">
+        <v>4270.99</v>
+      </c>
+      <c r="H107" s="20" t="n">
+        <v>4264.74</v>
+      </c>
+      <c r="I107" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J107" s="20" t="n">
+        <v>4281.98</v>
+      </c>
+      <c r="K107" s="23" t="n">
+        <v>7770</v>
+      </c>
+      <c r="L107" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M107" s="23" t="n">
+        <v>7769.95</v>
+      </c>
+      <c r="N107" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q107" s="24" t="inlineStr"/>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B108" s="20" t="inlineStr">
+        <is>
+          <t>20:43:28</t>
+        </is>
+      </c>
+      <c r="C108" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D108" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E108" s="20" t="n">
+        <v>4273.58</v>
+      </c>
+      <c r="F108" s="20" t="n">
+        <v>4286.9</v>
+      </c>
+      <c r="G108" s="20" t="n">
+        <v>4253.61</v>
+      </c>
+      <c r="H108" s="20" t="n">
+        <v>4246.95</v>
+      </c>
+      <c r="I108" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J108" s="20" t="n">
+        <v>4247.2</v>
+      </c>
+      <c r="K108" s="23" t="n">
+        <v>26380</v>
+      </c>
+      <c r="L108" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M108" s="23" t="n">
+        <v>26379.95</v>
+      </c>
+      <c r="N108" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q108" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7030,7 +7152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q89"/>
+  <dimension ref="A1:Q91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12398,6 +12520,128 @@
         </is>
       </c>
       <c r="Q89" s="19" t="inlineStr"/>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B90" s="20" t="inlineStr">
+        <is>
+          <t>18:27:09</t>
+        </is>
+      </c>
+      <c r="C90" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D90" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E90" s="20" t="n">
+        <v>4289.75</v>
+      </c>
+      <c r="F90" s="20" t="n">
+        <v>4302.26</v>
+      </c>
+      <c r="G90" s="20" t="n">
+        <v>4270.99</v>
+      </c>
+      <c r="H90" s="20" t="n">
+        <v>4264.74</v>
+      </c>
+      <c r="I90" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J90" s="20" t="n">
+        <v>4281.98</v>
+      </c>
+      <c r="K90" s="23" t="n">
+        <v>7770</v>
+      </c>
+      <c r="L90" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M90" s="23" t="n">
+        <v>7769.95</v>
+      </c>
+      <c r="N90" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q90" s="24" t="inlineStr"/>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B91" s="20" t="inlineStr">
+        <is>
+          <t>20:43:28</t>
+        </is>
+      </c>
+      <c r="C91" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E91" s="20" t="n">
+        <v>4273.58</v>
+      </c>
+      <c r="F91" s="20" t="n">
+        <v>4286.9</v>
+      </c>
+      <c r="G91" s="20" t="n">
+        <v>4253.61</v>
+      </c>
+      <c r="H91" s="20" t="n">
+        <v>4246.95</v>
+      </c>
+      <c r="I91" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J91" s="20" t="n">
+        <v>4247.2</v>
+      </c>
+      <c r="K91" s="23" t="n">
+        <v>26380</v>
+      </c>
+      <c r="L91" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M91" s="23" t="n">
+        <v>26379.95</v>
+      </c>
+      <c r="N91" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q91" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-29
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q108"/>
+  <dimension ref="A1:Q109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7136,6 +7136,67 @@
       </c>
       <c r="Q108" s="24" t="inlineStr"/>
     </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B109" s="20" t="inlineStr">
+        <is>
+          <t>01:13:05</t>
+        </is>
+      </c>
+      <c r="C109" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D109" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E109" s="20" t="n">
+        <v>4166.09</v>
+      </c>
+      <c r="F109" s="20" t="n">
+        <v>4153.3</v>
+      </c>
+      <c r="G109" s="20" t="n">
+        <v>4185.28</v>
+      </c>
+      <c r="H109" s="20" t="n">
+        <v>4191.67</v>
+      </c>
+      <c r="I109" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J109" s="20" t="n">
+        <v>4171.41</v>
+      </c>
+      <c r="K109" s="23" t="n">
+        <v>5320</v>
+      </c>
+      <c r="L109" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M109" s="23" t="n">
+        <v>5319.95</v>
+      </c>
+      <c r="N109" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q109" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7152,7 +7213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q91"/>
+  <dimension ref="A1:Q92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12642,6 +12703,67 @@
         </is>
       </c>
       <c r="Q91" s="24" t="inlineStr"/>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B92" s="20" t="inlineStr">
+        <is>
+          <t>01:13:05</t>
+        </is>
+      </c>
+      <c r="C92" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D92" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E92" s="20" t="n">
+        <v>4166.09</v>
+      </c>
+      <c r="F92" s="20" t="n">
+        <v>4153.3</v>
+      </c>
+      <c r="G92" s="20" t="n">
+        <v>4185.28</v>
+      </c>
+      <c r="H92" s="20" t="n">
+        <v>4191.67</v>
+      </c>
+      <c r="I92" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J92" s="20" t="n">
+        <v>4171.41</v>
+      </c>
+      <c r="K92" s="23" t="n">
+        <v>5320</v>
+      </c>
+      <c r="L92" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M92" s="23" t="n">
+        <v>5319.95</v>
+      </c>
+      <c r="N92" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q92" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-09-30
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q109"/>
+  <dimension ref="A1:Q110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7196,6 +7196,67 @@
         </is>
       </c>
       <c r="Q109" s="24" t="inlineStr"/>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C110" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E110" s="15" t="n">
+        <v>4154.27</v>
+      </c>
+      <c r="F110" s="15" t="n">
+        <v>4162.31</v>
+      </c>
+      <c r="G110" s="15" t="n">
+        <v>4142.22</v>
+      </c>
+      <c r="H110" s="15" t="n">
+        <v>4138.2</v>
+      </c>
+      <c r="I110" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J110" s="15" t="n">
+        <v>4155.29</v>
+      </c>
+      <c r="K110" s="18" t="n">
+        <v>-1015</v>
+      </c>
+      <c r="L110" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M110" s="18" t="n">
+        <v>-1015.05</v>
+      </c>
+      <c r="N110" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q110" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -13286,7 +13347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14079,6 +14140,67 @@
         </is>
       </c>
       <c r="Q14" s="19" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>4154.27</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>4162.31</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>4142.22</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>4138.2</v>
+      </c>
+      <c r="I15" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J15" s="15" t="n">
+        <v>4155.29</v>
+      </c>
+      <c r="K15" s="18" t="n">
+        <v>-1015</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M15" s="18" t="n">
+        <v>-1015.05</v>
+      </c>
+      <c r="N15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q15" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-01
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q110"/>
+  <dimension ref="A1:Q111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7258,6 +7258,67 @@
       </c>
       <c r="Q110" s="19" t="inlineStr"/>
     </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B111" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C111" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D111" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E111" s="20" t="n">
+        <v>4165.59</v>
+      </c>
+      <c r="F111" s="20" t="n">
+        <v>4149.96</v>
+      </c>
+      <c r="G111" s="20" t="n">
+        <v>4189.02</v>
+      </c>
+      <c r="H111" s="20" t="n">
+        <v>4196.84</v>
+      </c>
+      <c r="I111" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J111" s="20" t="n">
+        <v>4176.26</v>
+      </c>
+      <c r="K111" s="23" t="n">
+        <v>10675</v>
+      </c>
+      <c r="L111" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M111" s="23" t="n">
+        <v>10674.95</v>
+      </c>
+      <c r="N111" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q111" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7274,7 +7335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q92"/>
+  <dimension ref="A1:Q93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12825,6 +12886,67 @@
         </is>
       </c>
       <c r="Q92" s="24" t="inlineStr"/>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B93" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C93" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D93" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E93" s="20" t="n">
+        <v>4165.59</v>
+      </c>
+      <c r="F93" s="20" t="n">
+        <v>4149.96</v>
+      </c>
+      <c r="G93" s="20" t="n">
+        <v>4189.02</v>
+      </c>
+      <c r="H93" s="20" t="n">
+        <v>4196.84</v>
+      </c>
+      <c r="I93" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J93" s="20" t="n">
+        <v>4176.26</v>
+      </c>
+      <c r="K93" s="23" t="n">
+        <v>10675</v>
+      </c>
+      <c r="L93" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M93" s="23" t="n">
+        <v>10674.95</v>
+      </c>
+      <c r="N93" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q93" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-06
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q111"/>
+  <dimension ref="A1:Q113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7319,6 +7319,128 @@
       </c>
       <c r="Q111" s="24" t="inlineStr"/>
     </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B112" s="20" t="inlineStr">
+        <is>
+          <t>00:27:08</t>
+        </is>
+      </c>
+      <c r="C112" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D112" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E112" s="20" t="n">
+        <v>4152.81</v>
+      </c>
+      <c r="F112" s="20" t="n">
+        <v>4141.29</v>
+      </c>
+      <c r="G112" s="20" t="n">
+        <v>4170.09</v>
+      </c>
+      <c r="H112" s="20" t="n">
+        <v>4175.85</v>
+      </c>
+      <c r="I112" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J112" s="20" t="n">
+        <v>4176.6</v>
+      </c>
+      <c r="K112" s="23" t="n">
+        <v>23785</v>
+      </c>
+      <c r="L112" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M112" s="23" t="n">
+        <v>23784.95</v>
+      </c>
+      <c r="N112" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q112" s="24" t="inlineStr"/>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="inlineStr">
+        <is>
+          <t>01:19:47</t>
+        </is>
+      </c>
+      <c r="C113" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D113" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E113" s="15" t="n">
+        <v>4176.11</v>
+      </c>
+      <c r="F113" s="15" t="n">
+        <v>4167.61</v>
+      </c>
+      <c r="G113" s="15" t="n">
+        <v>4188.86</v>
+      </c>
+      <c r="H113" s="15" t="n">
+        <v>4193.11</v>
+      </c>
+      <c r="I113" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J113" s="15" t="n">
+        <v>4167.7</v>
+      </c>
+      <c r="K113" s="18" t="n">
+        <v>-8410</v>
+      </c>
+      <c r="L113" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M113" s="18" t="n">
+        <v>-8410.049999999999</v>
+      </c>
+      <c r="N113" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P113" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q113" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7335,7 +7457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q93"/>
+  <dimension ref="A1:Q95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12947,6 +13069,128 @@
         </is>
       </c>
       <c r="Q93" s="24" t="inlineStr"/>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B94" s="20" t="inlineStr">
+        <is>
+          <t>00:27:08</t>
+        </is>
+      </c>
+      <c r="C94" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D94" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E94" s="20" t="n">
+        <v>4152.81</v>
+      </c>
+      <c r="F94" s="20" t="n">
+        <v>4141.29</v>
+      </c>
+      <c r="G94" s="20" t="n">
+        <v>4170.09</v>
+      </c>
+      <c r="H94" s="20" t="n">
+        <v>4175.85</v>
+      </c>
+      <c r="I94" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J94" s="20" t="n">
+        <v>4176.6</v>
+      </c>
+      <c r="K94" s="23" t="n">
+        <v>23785</v>
+      </c>
+      <c r="L94" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M94" s="23" t="n">
+        <v>23784.95</v>
+      </c>
+      <c r="N94" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q94" s="24" t="inlineStr"/>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="inlineStr">
+        <is>
+          <t>01:19:47</t>
+        </is>
+      </c>
+      <c r="C95" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D95" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E95" s="15" t="n">
+        <v>4176.11</v>
+      </c>
+      <c r="F95" s="15" t="n">
+        <v>4167.61</v>
+      </c>
+      <c r="G95" s="15" t="n">
+        <v>4188.86</v>
+      </c>
+      <c r="H95" s="15" t="n">
+        <v>4193.11</v>
+      </c>
+      <c r="I95" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J95" s="15" t="n">
+        <v>4167.7</v>
+      </c>
+      <c r="K95" s="18" t="n">
+        <v>-8410</v>
+      </c>
+      <c r="L95" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M95" s="18" t="n">
+        <v>-8410.049999999999</v>
+      </c>
+      <c r="N95" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q95" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-07
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q113"/>
+  <dimension ref="A1:Q115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7441,6 +7441,128 @@
       </c>
       <c r="Q113" s="19" t="inlineStr"/>
     </row>
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C114" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D114" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E114" s="15" t="n">
+        <v>4102.65</v>
+      </c>
+      <c r="F114" s="15" t="n">
+        <v>4083.42</v>
+      </c>
+      <c r="G114" s="15" t="n">
+        <v>4131.48</v>
+      </c>
+      <c r="H114" s="15" t="n">
+        <v>4141.09</v>
+      </c>
+      <c r="I114" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J114" s="15" t="n">
+        <v>4101.44</v>
+      </c>
+      <c r="K114" s="18" t="n">
+        <v>-1205</v>
+      </c>
+      <c r="L114" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M114" s="18" t="n">
+        <v>-1205.05</v>
+      </c>
+      <c r="N114" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O114" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P114" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q114" s="19" t="inlineStr"/>
+    </row>
+    <row r="115" ht="20" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="inlineStr">
+        <is>
+          <t>01:56:34</t>
+        </is>
+      </c>
+      <c r="C115" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D115" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E115" s="15" t="n">
+        <v>4100.99</v>
+      </c>
+      <c r="F115" s="15" t="n">
+        <v>4111.37</v>
+      </c>
+      <c r="G115" s="15" t="n">
+        <v>4085.42</v>
+      </c>
+      <c r="H115" s="15" t="n">
+        <v>4080.24</v>
+      </c>
+      <c r="I115" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J115" s="15" t="n">
+        <v>4111.78</v>
+      </c>
+      <c r="K115" s="18" t="n">
+        <v>-10790</v>
+      </c>
+      <c r="L115" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M115" s="18" t="n">
+        <v>-10790.05</v>
+      </c>
+      <c r="N115" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O115" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P115" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q115" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7457,7 +7579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q95"/>
+  <dimension ref="A1:Q96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13191,6 +13313,67 @@
         </is>
       </c>
       <c r="Q95" s="19" t="inlineStr"/>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="inlineStr">
+        <is>
+          <t>01:56:34</t>
+        </is>
+      </c>
+      <c r="C96" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D96" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E96" s="15" t="n">
+        <v>4100.99</v>
+      </c>
+      <c r="F96" s="15" t="n">
+        <v>4111.37</v>
+      </c>
+      <c r="G96" s="15" t="n">
+        <v>4085.42</v>
+      </c>
+      <c r="H96" s="15" t="n">
+        <v>4080.24</v>
+      </c>
+      <c r="I96" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J96" s="15" t="n">
+        <v>4111.78</v>
+      </c>
+      <c r="K96" s="18" t="n">
+        <v>-10790</v>
+      </c>
+      <c r="L96" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M96" s="18" t="n">
+        <v>-10790.05</v>
+      </c>
+      <c r="N96" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q96" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -13713,7 +13896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14567,6 +14750,67 @@
         </is>
       </c>
       <c r="Q15" s="19" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>4102.65</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>4083.42</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>4131.48</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>4141.09</v>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J16" s="15" t="n">
+        <v>4101.44</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>-1205</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M16" s="18" t="n">
+        <v>-1205.05</v>
+      </c>
+      <c r="N16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q16" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-08
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q115"/>
+  <dimension ref="A1:Q116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7563,6 +7563,67 @@
       </c>
       <c r="Q115" s="19" t="inlineStr"/>
     </row>
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>23:20:30</t>
+        </is>
+      </c>
+      <c r="C116" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D116" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E116" s="15" t="n">
+        <v>4143.68</v>
+      </c>
+      <c r="F116" s="15" t="n">
+        <v>4128.14</v>
+      </c>
+      <c r="G116" s="15" t="n">
+        <v>4166.99</v>
+      </c>
+      <c r="H116" s="15" t="n">
+        <v>4174.77</v>
+      </c>
+      <c r="I116" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J116" s="15" t="n">
+        <v>4128.35</v>
+      </c>
+      <c r="K116" s="18" t="n">
+        <v>-15325</v>
+      </c>
+      <c r="L116" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M116" s="18" t="n">
+        <v>-15325.05</v>
+      </c>
+      <c r="N116" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P116" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q116" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7579,7 +7640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q96"/>
+  <dimension ref="A1:Q97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13374,6 +13435,67 @@
         </is>
       </c>
       <c r="Q96" s="19" t="inlineStr"/>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B97" s="15" t="inlineStr">
+        <is>
+          <t>23:20:30</t>
+        </is>
+      </c>
+      <c r="C97" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D97" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E97" s="15" t="n">
+        <v>4143.68</v>
+      </c>
+      <c r="F97" s="15" t="n">
+        <v>4128.14</v>
+      </c>
+      <c r="G97" s="15" t="n">
+        <v>4166.99</v>
+      </c>
+      <c r="H97" s="15" t="n">
+        <v>4174.77</v>
+      </c>
+      <c r="I97" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J97" s="15" t="n">
+        <v>4128.35</v>
+      </c>
+      <c r="K97" s="18" t="n">
+        <v>-15325</v>
+      </c>
+      <c r="L97" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M97" s="18" t="n">
+        <v>-15325.05</v>
+      </c>
+      <c r="N97" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P97" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q97" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-13
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q116"/>
+  <dimension ref="A1:Q117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7624,6 +7624,67 @@
       </c>
       <c r="Q116" s="19" t="inlineStr"/>
     </row>
+    <row r="117" ht="20" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="inlineStr">
+        <is>
+          <t>23:37:02</t>
+        </is>
+      </c>
+      <c r="C117" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D117" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E117" s="15" t="n">
+        <v>4149.99</v>
+      </c>
+      <c r="F117" s="15" t="n">
+        <v>4158.13</v>
+      </c>
+      <c r="G117" s="15" t="n">
+        <v>4137.79</v>
+      </c>
+      <c r="H117" s="15" t="n">
+        <v>4133.72</v>
+      </c>
+      <c r="I117" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J117" s="15" t="n">
+        <v>4158.92</v>
+      </c>
+      <c r="K117" s="18" t="n">
+        <v>-8925</v>
+      </c>
+      <c r="L117" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M117" s="18" t="n">
+        <v>-8925.049999999999</v>
+      </c>
+      <c r="N117" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O117" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P117" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q117" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7640,7 +7701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q97"/>
+  <dimension ref="A1:Q98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13496,6 +13557,67 @@
         </is>
       </c>
       <c r="Q97" s="19" t="inlineStr"/>
+    </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>23:37:02</t>
+        </is>
+      </c>
+      <c r="C98" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D98" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="n">
+        <v>4149.99</v>
+      </c>
+      <c r="F98" s="15" t="n">
+        <v>4158.13</v>
+      </c>
+      <c r="G98" s="15" t="n">
+        <v>4137.79</v>
+      </c>
+      <c r="H98" s="15" t="n">
+        <v>4133.72</v>
+      </c>
+      <c r="I98" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J98" s="15" t="n">
+        <v>4158.92</v>
+      </c>
+      <c r="K98" s="18" t="n">
+        <v>-8925</v>
+      </c>
+      <c r="L98" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M98" s="18" t="n">
+        <v>-8925.049999999999</v>
+      </c>
+      <c r="N98" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q98" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-15
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q117"/>
+  <dimension ref="A1:Q118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7685,6 +7685,67 @@
       </c>
       <c r="Q117" s="19" t="inlineStr"/>
     </row>
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B118" s="15" t="inlineStr">
+        <is>
+          <t>19:37:15</t>
+        </is>
+      </c>
+      <c r="C118" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D118" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E118" s="15" t="n">
+        <v>4161.4</v>
+      </c>
+      <c r="F118" s="15" t="n">
+        <v>4149.26</v>
+      </c>
+      <c r="G118" s="15" t="n">
+        <v>4179.6</v>
+      </c>
+      <c r="H118" s="15" t="n">
+        <v>4185.67</v>
+      </c>
+      <c r="I118" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J118" s="15" t="n">
+        <v>4150.32</v>
+      </c>
+      <c r="K118" s="18" t="n">
+        <v>-11080</v>
+      </c>
+      <c r="L118" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M118" s="18" t="n">
+        <v>-11080.05</v>
+      </c>
+      <c r="N118" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O118" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P118" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q118" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7701,7 +7762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q98"/>
+  <dimension ref="A1:Q99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13618,6 +13679,67 @@
         </is>
       </c>
       <c r="Q98" s="19" t="inlineStr"/>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B99" s="15" t="inlineStr">
+        <is>
+          <t>19:37:15</t>
+        </is>
+      </c>
+      <c r="C99" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D99" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E99" s="15" t="n">
+        <v>4161.4</v>
+      </c>
+      <c r="F99" s="15" t="n">
+        <v>4149.26</v>
+      </c>
+      <c r="G99" s="15" t="n">
+        <v>4179.6</v>
+      </c>
+      <c r="H99" s="15" t="n">
+        <v>4185.67</v>
+      </c>
+      <c r="I99" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J99" s="15" t="n">
+        <v>4150.32</v>
+      </c>
+      <c r="K99" s="18" t="n">
+        <v>-11080</v>
+      </c>
+      <c r="L99" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M99" s="18" t="n">
+        <v>-11080.05</v>
+      </c>
+      <c r="N99" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q99" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-20
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q118"/>
+  <dimension ref="A1:Q119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7746,6 +7746,67 @@
       </c>
       <c r="Q118" s="19" t="inlineStr"/>
     </row>
+    <row r="119" ht="20" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="inlineStr">
+        <is>
+          <t>19:09:54</t>
+        </is>
+      </c>
+      <c r="C119" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D119" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E119" s="15" t="n">
+        <v>4115.24</v>
+      </c>
+      <c r="F119" s="15" t="n">
+        <v>4126.37</v>
+      </c>
+      <c r="G119" s="15" t="n">
+        <v>4098.54</v>
+      </c>
+      <c r="H119" s="15" t="n">
+        <v>4092.98</v>
+      </c>
+      <c r="I119" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J119" s="15" t="n">
+        <v>4127.15</v>
+      </c>
+      <c r="K119" s="18" t="n">
+        <v>-11915</v>
+      </c>
+      <c r="L119" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M119" s="18" t="n">
+        <v>-11915.05</v>
+      </c>
+      <c r="N119" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P119" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q119" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7762,7 +7823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q99"/>
+  <dimension ref="A1:Q100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13740,6 +13801,67 @@
         </is>
       </c>
       <c r="Q99" s="19" t="inlineStr"/>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B100" s="15" t="inlineStr">
+        <is>
+          <t>19:09:54</t>
+        </is>
+      </c>
+      <c r="C100" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D100" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E100" s="15" t="n">
+        <v>4115.24</v>
+      </c>
+      <c r="F100" s="15" t="n">
+        <v>4126.37</v>
+      </c>
+      <c r="G100" s="15" t="n">
+        <v>4098.54</v>
+      </c>
+      <c r="H100" s="15" t="n">
+        <v>4092.98</v>
+      </c>
+      <c r="I100" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J100" s="15" t="n">
+        <v>4127.15</v>
+      </c>
+      <c r="K100" s="18" t="n">
+        <v>-11915</v>
+      </c>
+      <c r="L100" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M100" s="18" t="n">
+        <v>-11915.05</v>
+      </c>
+      <c r="N100" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P100" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q100" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-21
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q119"/>
+  <dimension ref="A1:Q120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7807,6 +7807,67 @@
       </c>
       <c r="Q119" s="19" t="inlineStr"/>
     </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
+        <is>
+          <t>00:26:27</t>
+        </is>
+      </c>
+      <c r="C120" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D120" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E120" s="15" t="n">
+        <v>4132.35</v>
+      </c>
+      <c r="F120" s="15" t="n">
+        <v>4122</v>
+      </c>
+      <c r="G120" s="15" t="n">
+        <v>4147.86</v>
+      </c>
+      <c r="H120" s="15" t="n">
+        <v>4153.04</v>
+      </c>
+      <c r="I120" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J120" s="15" t="n">
+        <v>4121.68</v>
+      </c>
+      <c r="K120" s="18" t="n">
+        <v>-10670</v>
+      </c>
+      <c r="L120" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M120" s="18" t="n">
+        <v>-10670.05</v>
+      </c>
+      <c r="N120" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O120" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P120" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q120" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7823,7 +7884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q100"/>
+  <dimension ref="A1:Q101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13862,6 +13923,67 @@
         </is>
       </c>
       <c r="Q100" s="19" t="inlineStr"/>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B101" s="15" t="inlineStr">
+        <is>
+          <t>00:26:27</t>
+        </is>
+      </c>
+      <c r="C101" s="25" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D101" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E101" s="15" t="n">
+        <v>4132.35</v>
+      </c>
+      <c r="F101" s="15" t="n">
+        <v>4122</v>
+      </c>
+      <c r="G101" s="15" t="n">
+        <v>4147.86</v>
+      </c>
+      <c r="H101" s="15" t="n">
+        <v>4153.04</v>
+      </c>
+      <c r="I101" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J101" s="15" t="n">
+        <v>4121.68</v>
+      </c>
+      <c r="K101" s="18" t="n">
+        <v>-10670</v>
+      </c>
+      <c r="L101" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M101" s="18" t="n">
+        <v>-10670.05</v>
+      </c>
+      <c r="N101" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q101" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-22
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q120"/>
+  <dimension ref="A1:Q121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7867,6 +7867,67 @@
         </is>
       </c>
       <c r="Q120" s="19" t="inlineStr"/>
+    </row>
+    <row r="121" ht="20" customHeight="1">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="inlineStr">
+        <is>
+          <t>22:18:30</t>
+        </is>
+      </c>
+      <c r="C121" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D121" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E121" s="15" t="n">
+        <v>4055.85</v>
+      </c>
+      <c r="F121" s="15" t="n">
+        <v>4037.92</v>
+      </c>
+      <c r="G121" s="15" t="n">
+        <v>4082.73</v>
+      </c>
+      <c r="H121" s="15" t="n">
+        <v>4091.69</v>
+      </c>
+      <c r="I121" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J121" s="15" t="n">
+        <v>4035.03</v>
+      </c>
+      <c r="K121" s="18" t="n">
+        <v>-20810</v>
+      </c>
+      <c r="L121" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M121" s="18" t="n">
+        <v>-20810.05</v>
+      </c>
+      <c r="N121" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O121" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P121" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q121" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -14506,7 +14567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15421,6 +15482,67 @@
         </is>
       </c>
       <c r="Q16" s="19" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>22:18:30</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>4055.85</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>4037.92</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>4082.73</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <v>4091.69</v>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J17" s="15" t="n">
+        <v>4035.03</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <v>-20810</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M17" s="18" t="n">
+        <v>-20810.05</v>
+      </c>
+      <c r="N17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q17" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-27
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q121"/>
+  <dimension ref="A1:Q122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7929,6 +7929,67 @@
       </c>
       <c r="Q121" s="19" t="inlineStr"/>
     </row>
+    <row r="122" ht="20" customHeight="1">
+      <c r="A122" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B122" s="20" t="inlineStr">
+        <is>
+          <t>20:27:27</t>
+        </is>
+      </c>
+      <c r="C122" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D122" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E122" s="20" t="n">
+        <v>4030.53</v>
+      </c>
+      <c r="F122" s="20" t="n">
+        <v>4018.62</v>
+      </c>
+      <c r="G122" s="20" t="n">
+        <v>4048.39</v>
+      </c>
+      <c r="H122" s="20" t="n">
+        <v>4054.35</v>
+      </c>
+      <c r="I122" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J122" s="20" t="n">
+        <v>4051.42</v>
+      </c>
+      <c r="K122" s="23" t="n">
+        <v>20890</v>
+      </c>
+      <c r="L122" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M122" s="23" t="n">
+        <v>20889.95</v>
+      </c>
+      <c r="N122" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P122" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q122" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -7945,7 +8006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q101"/>
+  <dimension ref="A1:Q102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14045,6 +14106,67 @@
         </is>
       </c>
       <c r="Q101" s="19" t="inlineStr"/>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B102" s="20" t="inlineStr">
+        <is>
+          <t>20:27:27</t>
+        </is>
+      </c>
+      <c r="C102" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D102" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E102" s="20" t="n">
+        <v>4030.53</v>
+      </c>
+      <c r="F102" s="20" t="n">
+        <v>4018.62</v>
+      </c>
+      <c r="G102" s="20" t="n">
+        <v>4048.39</v>
+      </c>
+      <c r="H102" s="20" t="n">
+        <v>4054.35</v>
+      </c>
+      <c r="I102" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J102" s="20" t="n">
+        <v>4051.42</v>
+      </c>
+      <c r="K102" s="23" t="n">
+        <v>20890</v>
+      </c>
+      <c r="L102" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M102" s="23" t="n">
+        <v>20889.95</v>
+      </c>
+      <c r="N102" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q102" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 NY session — 2026-10-28
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q122"/>
+  <dimension ref="A1:Q123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7990,6 +7990,67 @@
       </c>
       <c r="Q122" s="24" t="inlineStr"/>
     </row>
+    <row r="123" ht="20" customHeight="1">
+      <c r="A123" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B123" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C123" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D123" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E123" s="20" t="n">
+        <v>4059.28</v>
+      </c>
+      <c r="F123" s="20" t="n">
+        <v>4053.28</v>
+      </c>
+      <c r="G123" s="20" t="n">
+        <v>4068.26</v>
+      </c>
+      <c r="H123" s="20" t="n">
+        <v>4071.26</v>
+      </c>
+      <c r="I123" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J123" s="20" t="n">
+        <v>4061.1</v>
+      </c>
+      <c r="K123" s="23" t="n">
+        <v>1825</v>
+      </c>
+      <c r="L123" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M123" s="23" t="n">
+        <v>1824.95</v>
+      </c>
+      <c r="N123" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P123" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q123" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -8006,7 +8067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q102"/>
+  <dimension ref="A1:Q103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14167,6 +14228,67 @@
         </is>
       </c>
       <c r="Q102" s="24" t="inlineStr"/>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B103" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C103" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D103" s="23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E103" s="20" t="n">
+        <v>4059.28</v>
+      </c>
+      <c r="F103" s="20" t="n">
+        <v>4053.28</v>
+      </c>
+      <c r="G103" s="20" t="n">
+        <v>4068.26</v>
+      </c>
+      <c r="H103" s="20" t="n">
+        <v>4071.26</v>
+      </c>
+      <c r="I103" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J103" s="20" t="n">
+        <v>4061.1</v>
+      </c>
+      <c r="K103" s="23" t="n">
+        <v>1825</v>
+      </c>
+      <c r="L103" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M103" s="23" t="n">
+        <v>1824.95</v>
+      </c>
+      <c r="N103" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q103" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-28
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q123"/>
+  <dimension ref="A1:Q125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8051,6 +8051,128 @@
       </c>
       <c r="Q123" s="24" t="inlineStr"/>
     </row>
+    <row r="124" ht="20" customHeight="1">
+      <c r="A124" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B124" s="20" t="inlineStr">
+        <is>
+          <t>00:03:31</t>
+        </is>
+      </c>
+      <c r="C124" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D124" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E124" s="20" t="n">
+        <v>4043.49</v>
+      </c>
+      <c r="F124" s="20" t="n">
+        <v>4050.86</v>
+      </c>
+      <c r="G124" s="20" t="n">
+        <v>4032.44</v>
+      </c>
+      <c r="H124" s="20" t="n">
+        <v>4028.76</v>
+      </c>
+      <c r="I124" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J124" s="20" t="n">
+        <v>4026.77</v>
+      </c>
+      <c r="K124" s="23" t="n">
+        <v>16715</v>
+      </c>
+      <c r="L124" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M124" s="23" t="n">
+        <v>16714.95</v>
+      </c>
+      <c r="N124" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P124" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q124" s="24" t="inlineStr"/>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B125" s="15" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C125" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D125" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E125" s="15" t="n">
+        <v>4052.97</v>
+      </c>
+      <c r="F125" s="15" t="n">
+        <v>4072.07</v>
+      </c>
+      <c r="G125" s="15" t="n">
+        <v>4024.31</v>
+      </c>
+      <c r="H125" s="15" t="n">
+        <v>4014.76</v>
+      </c>
+      <c r="I125" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J125" s="15" t="n">
+        <v>4063.16</v>
+      </c>
+      <c r="K125" s="18" t="n">
+        <v>-10190</v>
+      </c>
+      <c r="L125" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M125" s="18" t="n">
+        <v>-10190.05</v>
+      </c>
+      <c r="N125" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P125" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q125" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -8067,7 +8189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q103"/>
+  <dimension ref="A1:Q104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14289,6 +14411,67 @@
         </is>
       </c>
       <c r="Q103" s="24" t="inlineStr"/>
+    </row>
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B104" s="20" t="inlineStr">
+        <is>
+          <t>00:03:31</t>
+        </is>
+      </c>
+      <c r="C104" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D104" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E104" s="20" t="n">
+        <v>4043.49</v>
+      </c>
+      <c r="F104" s="20" t="n">
+        <v>4050.86</v>
+      </c>
+      <c r="G104" s="20" t="n">
+        <v>4032.44</v>
+      </c>
+      <c r="H104" s="20" t="n">
+        <v>4028.76</v>
+      </c>
+      <c r="I104" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J104" s="20" t="n">
+        <v>4026.77</v>
+      </c>
+      <c r="K104" s="23" t="n">
+        <v>16715</v>
+      </c>
+      <c r="L104" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M104" s="23" t="n">
+        <v>16714.95</v>
+      </c>
+      <c r="N104" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P104" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q104" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -14811,7 +14994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15787,6 +15970,67 @@
         </is>
       </c>
       <c r="Q17" s="19" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>S3 Silver Bullet</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>4052.97</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>4072.07</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>4024.31</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <v>4014.76</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J18" s="15" t="n">
+        <v>4063.16</v>
+      </c>
+      <c r="K18" s="18" t="n">
+        <v>-10190</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M18" s="18" t="n">
+        <v>-10190.05</v>
+      </c>
+      <c r="N18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="18" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q18" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
📊 London session — 2026-10-29
</commit_message>
<xml_diff>
--- a/xauusd_trades.xlsx
+++ b/xauusd_trades.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q125"/>
+  <dimension ref="A1:Q126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8173,6 +8173,67 @@
       </c>
       <c r="Q125" s="19" t="inlineStr"/>
     </row>
+    <row r="126" ht="20" customHeight="1">
+      <c r="A126" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B126" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C126" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D126" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E126" s="20" t="n">
+        <v>4024.53</v>
+      </c>
+      <c r="F126" s="20" t="n">
+        <v>4039.44</v>
+      </c>
+      <c r="G126" s="20" t="n">
+        <v>4002.16</v>
+      </c>
+      <c r="H126" s="20" t="n">
+        <v>3994.71</v>
+      </c>
+      <c r="I126" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J126" s="20" t="n">
+        <v>4021.93</v>
+      </c>
+      <c r="K126" s="23" t="n">
+        <v>2600</v>
+      </c>
+      <c r="L126" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M126" s="23" t="n">
+        <v>2599.95</v>
+      </c>
+      <c r="N126" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P126" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q126" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -8189,7 +8250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q104"/>
+  <dimension ref="A1:Q105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14472,6 +14533,67 @@
         </is>
       </c>
       <c r="Q104" s="24" t="inlineStr"/>
+    </row>
+    <row r="105" ht="20" customHeight="1">
+      <c r="A105" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B105" s="20" t="inlineStr">
+        <is>
+          <t>01:25:01</t>
+        </is>
+      </c>
+      <c r="C105" s="21" t="inlineStr">
+        <is>
+          <t>S1 Asian Breakout</t>
+        </is>
+      </c>
+      <c r="D105" s="22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E105" s="20" t="n">
+        <v>4024.53</v>
+      </c>
+      <c r="F105" s="20" t="n">
+        <v>4039.44</v>
+      </c>
+      <c r="G105" s="20" t="n">
+        <v>4002.16</v>
+      </c>
+      <c r="H105" s="20" t="n">
+        <v>3994.71</v>
+      </c>
+      <c r="I105" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="J105" s="20" t="n">
+        <v>4021.93</v>
+      </c>
+      <c r="K105" s="23" t="n">
+        <v>2600</v>
+      </c>
+      <c r="L105" s="20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M105" s="23" t="n">
+        <v>2599.95</v>
+      </c>
+      <c r="N105" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" s="23" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q105" s="24" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>